<commit_message>
feat: add full PowerPoint and PDF reports, Tufte charts, and Framsikt/Net Zero Power BI and Excel model updates
</commit_message>
<xml_diff>
--- a/Kristiansand_EPM_Excel_Modell.xlsx
+++ b/Kristiansand_EPM_Excel_Modell.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Konsern_Styringsrapport" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Mevold_Grunnskole" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Slettheia_Bofellesskap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_EOY_Prognosemodell" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Net_Zero_Tiltaksplan" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Audit_AI_HITL" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fact_Regnskap" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dim_Funksjon" sheetId="7" state="visible" r:id="rId7"/>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="#,##0 kr"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +90,13 @@
       <color rgb="00C53030"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002B6CB0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +119,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F7FAFC"/>
         <bgColor rgb="00F7FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
       </patternFill>
     </fill>
   </fills>
@@ -254,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -301,7 +312,21 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1828,447 +1853,783 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="47" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>MEVOLD GRUNNSKOLE - RAMMESTYRING &amp; AVVIK (KOSTRA 202)</t>
+          <t>MEVOLD GRUNNSKOLE - RAMMESTYRING &amp; ENHETSFORDELING (KOSTRA 202)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Oppvekstsektoren | Rektor Mevold Grunnskole | YTD per August 2025</t>
+          <t>Oppvekstsektoren | Rektor Mevold Grunnskole | Framsikt visning (jfr. skole1.png og skole_framsikt_cond_format.png)</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Art Kode</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Kostnadspost / Art</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Kategori</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
-        <is>
-          <t>Budsjett YTD (kr)</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Regnskap YTD (kr)</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. ENHETSFORDELING PER 2. TERTIAL (FRAMSIKT MATRISE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Enhet (brukt)</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Regnskap hiå (kr)</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Budsjett hiå (kr)</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Avvik i kr</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>Avvik %</t>
         </is>
       </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>Diagnose &amp; Tiltak</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>1010</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>1010 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="n">
-        <v>9782000</v>
-      </c>
-      <c r="F6" s="17" t="n">
-        <v>10999000</v>
-      </c>
-      <c r="G6" s="18" t="n">
-        <v>1217000</v>
-      </c>
-      <c r="H6" s="19" t="n">
-        <v>0.1244121856471069</v>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak B: Optimalisere assistentdekning</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>1020</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>1020 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="n">
-        <v>101000</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>583000</v>
-      </c>
-      <c r="G7" s="18" t="n">
-        <v>482000</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>4.772277227722772</v>
-      </c>
-      <c r="I7" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak B: Optimalisere assistentdekning</t>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Årsbudsjett (kr)</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Brukt hiå %</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>KPI Status</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>1090</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>1090 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="n">
-        <v>2182000</v>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>2433000</v>
-      </c>
-      <c r="G8" s="18" t="n">
-        <v>251000</v>
+          <t>Ordinær undervisning</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>12024000</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>11385000</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>-639000</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>-0.056</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>17590000</v>
       </c>
       <c r="H8" s="19" t="n">
-        <v>0.115032080659945</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>Tiltak B: Optimalisere assistentdekning</t>
+          <t>🚩 Merforbruk</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>1690</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>1690 Kompensasjon moms påløpt i driftsregnskapet</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Refusjon</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="17" t="n">
-        <v>194000</v>
-      </c>
-      <c r="G9" s="18" t="n">
-        <v>194000</v>
+          <t>Spesialundervisning grunnskole</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>2792000</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>2496000</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>-296000</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>-0.119</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>4114000</v>
       </c>
       <c r="H9" s="19" t="n">
-        <v>0</v>
+        <v>0.679</v>
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>Tiltak A: Avstemme sykelønnsrefusjon mot NAV</t>
+          <t>🚩 Merforbruk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>1040</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>1040 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
+          <t>Grunnskole (felles)</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>1733000</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>1761000</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F10" s="17" t="n">
-        <v>166000</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>147000</v>
+        <v>28000</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>2919000</v>
       </c>
       <c r="H10" s="19" t="n">
-        <v>7.736842105263158</v>
+        <v>0.594</v>
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>Tiltak B: Optimalisere assistentdekning</t>
+          <t>✓ Under ramme</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>1030</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>1030 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>97000</v>
-      </c>
-      <c r="G11" s="18" t="n">
-        <v>97000</v>
+          <t>Skolefritidstilbud (SFO)</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>983000</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>813000</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>-170000</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>-0.209</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>1233000</v>
       </c>
       <c r="H11" s="19" t="n">
-        <v>0</v>
+        <v>0.797</v>
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>Tiltak B: Optimalisere assistentdekning</t>
+          <t>🚩 Merforbruk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>1130</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>1130 11 Refusjon lønn</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>Refusjon</t>
-        </is>
+          <t>Voksenopplæring</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>491000</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>513000</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>151000</v>
-      </c>
-      <c r="F12" s="17" t="n">
-        <v>201000</v>
-      </c>
-      <c r="G12" s="18" t="n">
-        <v>50000</v>
+        <v>22000</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>35000</v>
       </c>
       <c r="H12" s="19" t="n">
-        <v>0.3311258278145696</v>
+        <v>14.029</v>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>Tiltak A: Avstemme sykelønnsrefusjon mot NAV</t>
+          <t>Avstemmes</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>1270</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>1270 11 Refusjon lønn</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>Refusjon</t>
-        </is>
+          <t>Skoleskyss</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>469000</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>516000</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="17" t="n">
-        <v>39000</v>
-      </c>
-      <c r="G13" s="18" t="n">
-        <v>39000</v>
+        <v>47000</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>775000</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>0</v>
+        <v>0.605</v>
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>Tiltak A: Avstemme sykelønnsrefusjon mot NAV</t>
+          <t>✓ Under ramme</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>1110</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>1110 11 Refusjon lønn</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>Refusjon</t>
-        </is>
+          <t>PPT (Pedagogisk-psykologisk)</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>286000</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>350000</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>143000</v>
-      </c>
-      <c r="F14" s="17" t="n">
-        <v>135000</v>
+        <v>64000</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0.183</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>-8000</v>
+        <v>700000</v>
       </c>
       <c r="H14" s="19" t="n">
-        <v>-0.05594405594405594</v>
+        <v>0.409</v>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Tiltak A: Avstemme sykelønnsrefusjon mot NAV</t>
+          <t>✓ Under ramme</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="16" t="inlineStr">
         <is>
+          <t>Ekskursjonar / Leirskule</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>124000</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>124000</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>124000</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>I balanse</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>TOTALT MEVOLD GRUNNSKOLE</t>
+        </is>
+      </c>
+      <c r="C16" s="22">
+        <f>SUM(C8:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="22">
+        <f>SUM(D8:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="22">
+        <f>SUM(E8:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>IF(D16&gt;0, E16/D16, 0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="22">
+        <f>SUM(G8:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="23">
+        <f>IF(G16&gt;0, C16/G16, 0)</f>
+        <v/>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>🚩 Samlet merforbruk</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>2. HOVEDPOSTER &amp; DIAGNOSE (KOSTRA ARTER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Art Kode</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Kostnadspost / Art</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Budsjett YTD (kr)</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Regnskap YTD (kr)</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Avvik i kr</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Avvik %</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>Diagnose &amp; Tiltak</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>1010</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>1010 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>9782000</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>10999000</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <v>1217000</v>
+      </c>
+      <c r="H22" s="19" t="n">
+        <v>0.1244121856471069</v>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S1: Vikarstopp &amp; timeplanjustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>1020</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>1020 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>101000</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>583000</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>482000</v>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>4.772277227722772</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S1: Vikarstopp &amp; timeplanjustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>1090</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>1090 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>2182000</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>2433000</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <v>251000</v>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>0.115032080659945</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S1: Vikarstopp &amp; timeplanjustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>1690</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>1690 Kompensasjon moms påløpt i driftsregnskapet</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Refusjon</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>194000</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>194000</v>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S4: Avstemme sykelønnsrefusjon mot NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>1040 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>166000</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <v>147000</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>7.736842105263158</v>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S1: Vikarstopp &amp; timeplanjustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>1030</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>1030 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>97000</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>97000</v>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S1: Vikarstopp &amp; timeplanjustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>1130</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>1130 11 Refusjon lønn</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Refusjon</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>151000</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>201000</v>
+      </c>
+      <c r="G28" s="18" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>0.3311258278145696</v>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S4: Avstemme sykelønnsrefusjon mot NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>1270</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>1270 11 Refusjon lønn</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Refusjon</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>39000</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>39000</v>
+      </c>
+      <c r="H29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S4: Avstemme sykelønnsrefusjon mot NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>1110</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>1110 11 Refusjon lønn</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Refusjon</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="n">
+        <v>143000</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>135000</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="H30" s="19" t="n">
+        <v>-0.05594405594405594</v>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S4: Avstemme sykelønnsrefusjon mot NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
           <t>1150</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>1150 11 Refusjon lønn</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Refusjon</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E31" s="17" t="n">
         <v>753000</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F31" s="17" t="n">
         <v>637000</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G31" s="17" t="n">
         <v>-116000</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H31" s="19" t="n">
         <v>-0.1540504648074369</v>
       </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak A: Avstemme sykelønnsrefusjon mot NAV</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="16" t="inlineStr">
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak S4: Avstemme sykelønnsrefusjon mot NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>1050</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>1050 10 Lønn</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E32" s="17" t="n">
         <v>15000</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F32" s="17" t="n">
         <v>-1339000</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G32" s="17" t="n">
         <v>-1354000</v>
       </c>
-      <c r="H16" s="19" t="n">
+      <c r="H32" s="19" t="n">
         <v>-90.26666666666667</v>
       </c>
-      <c r="I16" s="16" t="inlineStr">
+      <c r="I32" s="16" t="inlineStr">
         <is>
           <t>I henhold til ramme</t>
         </is>
@@ -2285,16 +2646,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
@@ -2310,7 +2671,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Helse og mestring | Enhetsleder Slettheia | Januar-Desember 2024</t>
+          <t>Helse og mestring | Enhetsleder Slettheia | Framsikt visning (jfr. boom1.png og boom2.png)</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2679,7 @@
     <row r="5">
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>TOPP KOSTNADSDRIVERE (YTD JANUAR-AUGUST)</t>
+          <t>1. MÅNEDLIG AVVIKSUTVIKLING JANUAR-AUGUST (BOOM1.PNG)</t>
         </is>
       </c>
     </row>
@@ -2326,450 +2687,644 @@
     <row r="7">
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Kontokode</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Kontonavn</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>KOSTRA Art</t>
+          <t>Måned</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Budsjett (kr)</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Regnskap (kr)</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>Budsjett YTD (kr)</t>
+          <t>Avvik i kr</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Regnskap YTD (kr)</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
-        <is>
-          <t>Merforbruk i kr</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
-        <is>
-          <t>Merforbruk %</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>Rotårsak &amp; Tiltaksmeny</t>
+          <t>Avvik %</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Hendelse / Avviksdiagnose</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>1710</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>1710 11 Refusjon lønn</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>1710</t>
-        </is>
+          <t>Januar</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>1403337</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>1014752</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>-716385</v>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>732705</v>
-      </c>
-      <c r="G8" s="18" t="n">
-        <v>1449090</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak B: Søke toppfinansiering ressurskrevende brukere</t>
+        <v>388585</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Stabil grunnbemanning, lavt vikarinnleie</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>1020</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>1020 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>1020</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>856632</v>
-      </c>
-      <c r="F9" s="17" t="n">
-        <v>1224900</v>
-      </c>
-      <c r="G9" s="18" t="n">
-        <v>368268</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>0.4299022217241476</v>
-      </c>
-      <c r="I9" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak B: Søke toppfinansiering ressurskrevende brukere</t>
+          <t>Februar</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>1410893</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>2082090</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>-671197</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>-0.476</v>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>🚨 Februarsjokk: Akutt influensatopp, overtid og eksterne vikarbyråer</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>1030</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>1030 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>1030</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="17" t="n">
-        <v>209540</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>209540</v>
-      </c>
-      <c r="H10" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Tiltak B: Søke toppfinansiering ressurskrevende brukere</t>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>1342381</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>1541249</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>-198868</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>-0.148</v>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>Etterslep i sykefravær og høyt nattillegg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>1010</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>1010 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>1010</t>
-        </is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>2357359</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>2256716</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>7172914</v>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>7368070</v>
-      </c>
-      <c r="G11" s="18" t="n">
-        <v>195156</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>0.02720735254876888</v>
-      </c>
-      <c r="I11" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
+        <v>100643</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Feriepengeavstemming og refusjoner</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>1040</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>1040 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>1040</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>56504</v>
-      </c>
-      <c r="F12" s="17" t="n">
-        <v>242076</v>
-      </c>
-      <c r="G12" s="18" t="n">
-        <v>185572</v>
-      </c>
-      <c r="H12" s="19" t="n">
-        <v>3.284227665298032</v>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
+          <t>Mai</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>1544215</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>1613437</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>-69222</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>-0.045</v>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Stabilt merforbruk knyttet til 2:1-vedtak</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>1050</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>1050 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>1050</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>13992</v>
-      </c>
-      <c r="F13" s="17" t="n">
-        <v>125046</v>
-      </c>
-      <c r="G13" s="18" t="n">
-        <v>111054</v>
-      </c>
-      <c r="H13" s="19" t="n">
-        <v>7.936963979416809</v>
-      </c>
-      <c r="I13" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
+          <t>Juni</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>241681</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>519336</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>-277655</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>-1.149</v>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Sommerturnusstart, lavt budsjettgrunnlag</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>1099</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>1099 10 Lønn</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>1099</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="n">
-        <v>1425817</v>
-      </c>
-      <c r="F14" s="17" t="n">
-        <v>1527431</v>
-      </c>
-      <c r="G14" s="18" t="n">
-        <v>101614</v>
-      </c>
-      <c r="H14" s="19" t="n">
-        <v>0.07126721030819523</v>
-      </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
+          <t>Juli</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>1512209</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>1837523</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>-325314</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>-0.215</v>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Bruk av eksternt vikarbyrå i fellesferien</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="16" t="inlineStr">
         <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>1525162</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>1765810</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>-240648</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>-0.158</v>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Siste avsluttede måned: Høyt kvelds-/helgepress</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>YTD T2 AKKUMULERT</t>
+        </is>
+      </c>
+      <c r="C16" s="22">
+        <f>SUM(C8:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="22">
+        <f>SUM(D8:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="22">
+        <f>SUM(E8:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>IF(C16&gt;0, E16/C16, 0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Akkumulert overforbruk som krever korrigering</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>2. TOPP KOSTNADSDRIVERE (ARTERYTD JANUAR-AUGUST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Kontokode</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Kontonavn</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>KOSTRA Art</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Budsjett YTD (kr)</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Regnskap YTD (kr)</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Merforbruk i kr</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Merforbruk %</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>Rotårsak &amp; Tiltaksmeny</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>1710</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>1710 11 Refusjon lønn</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>1710</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>-716385</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>732705</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <v>1449090</v>
+      </c>
+      <c r="H22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B5: Søke toppfinansiering ressurskrevende brukere</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>1020</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>1020 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>1020</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>856632</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>1224900</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>368268</v>
+      </c>
+      <c r="H23" s="19" t="n">
+        <v>0.4299022217241476</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B5: Søke toppfinansiering ressurskrevende brukere</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>1030</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>1030 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>1030</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>209540</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <v>209540</v>
+      </c>
+      <c r="H24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B5: Søke toppfinansiering ressurskrevende brukere</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>1010</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>1010 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>1010</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>7172914</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>7368070</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>195156</v>
+      </c>
+      <c r="H25" s="19" t="n">
+        <v>0.02720735254876888</v>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>1040 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>56504</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>242076</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <v>185572</v>
+      </c>
+      <c r="H26" s="19" t="n">
+        <v>3.284227665298032</v>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>1050 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>13992</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>125046</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>111054</v>
+      </c>
+      <c r="H27" s="19" t="n">
+        <v>7.936963979416809</v>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>1099</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>1099 10 Lønn</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>1099</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>1425817</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>1527431</v>
+      </c>
+      <c r="G28" s="18" t="n">
+        <v>101614</v>
+      </c>
+      <c r="H28" s="19" t="n">
+        <v>0.07126721030819523</v>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="16" t="inlineStr">
+        <is>
           <t>1729</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>1729 14 Overføringer</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>1729</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E29" s="17" t="n">
         <v>-93296</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F29" s="17" t="n">
         <v>-35217</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G29" s="18" t="n">
         <v>58079</v>
       </c>
-      <c r="H15" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="16" t="inlineStr">
+      <c r="H29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>1120</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>1120 11 Refusjon lønn</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>1120</t>
         </is>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E30" s="17" t="n">
         <v>69056</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F30" s="17" t="n">
         <v>103020</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G30" s="17" t="n">
         <v>33964</v>
       </c>
-      <c r="H16" s="19" t="n">
+      <c r="H30" s="19" t="n">
         <v>0.4918327154772938</v>
       </c>
-      <c r="I16" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>1700 17 Refusjoner</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>1700</t>
         </is>
       </c>
-      <c r="E17" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="17" t="n">
+      <c r="E31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="17" t="n">
         <v>7100</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G31" s="17" t="n">
         <v>7100</v>
       </c>
-      <c r="H17" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>1770</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>1770 17 Refusjoner</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>1770</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="17" t="n">
-        <v>960</v>
-      </c>
-      <c r="G18" s="17" t="n">
-        <v>960</v>
-      </c>
-      <c r="H18" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>1500 15 Finansutgifter</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="G19" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="H19" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <t>Turnusjustering T3</t>
+      <c r="H31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Tiltak B2: Turnusomlegging T3</t>
         </is>
       </c>
     </row>
@@ -2784,41 +3339,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>RULLENDE EOY-PROGNOSE &amp; SENSITIVITETSANALYSE</t>
+          <t>KORRIGERENDE TILTAKSMATRISE &amp; NET ZERO BALANSERING</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Prognosemodell forventet årsavvik jf. Kommuneloven § 14-5 (Varslingsplikt)</t>
+          <t>Konkrete innsparingstiltak i T3 (Sept-Des) for å oppnå 0 kr i helårsavvik jf. Kommuneloven § 14-5</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Formel: EOY Prognose = Regnskap YTD + Gjenstående Budsjett + (Avvik YTD * Trendfaktor)</t>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. EOY PROGNOSE OG NET ZERO LUKKING</t>
         </is>
       </c>
     </row>
@@ -2826,184 +3380,588 @@
     <row r="7">
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Enhet / Ansvar</t>
+          <t>Enhet / Virksomhetsområde</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Budsjett YTD (kr)</t>
+          <t>Vedtatt Årsbudsjett</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Regnskap YTD (kr)</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="inlineStr">
-        <is>
-          <t>Avvik YTD (kr)</t>
+          <t>Regnskap YTD (T2)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Run-Rate EOY (Uendret)</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Restbudsjett T3 (kr)</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>Vedtatt Årsbudsjett</t>
+          <t>Uavbøtt Avvik EOY</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Tiltak T3 (Sept-Des)</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>Trendfaktor</t>
-        </is>
-      </c>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>EOY Prognose (kr)</t>
-        </is>
-      </c>
-      <c r="J7" s="15" t="inlineStr">
-        <is>
-          <t>Forventet Årsavvik (kr)</t>
+          <t>EOY Regnskap m/ Tiltak</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>Sluttavvik 31.12 (Mål)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Mevold Grunnskole (Oppvekst)</t>
+          <t>Slettheia Bofellesskap (Helse)</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>13146000</v>
+        <v>17233691</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>14145000</v>
-      </c>
-      <c r="E8" s="17">
-        <f>D8-C8</f>
-        <v/>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>13146000</v>
-      </c>
-      <c r="H8" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I8" s="17">
-        <f>D8+F8+(E8*H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="18">
-        <f>I8-G8</f>
-        <v/>
+        <v>12622851</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>19162112</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>-1928421</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>1928421</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>17233691</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Slettheia Bofellesskap (Helse)</t>
+          <t>Mevold Grunnskole (Oppvekst)</t>
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>11337237</v>
+        <v>27490000</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>12622851</v>
-      </c>
-      <c r="E9" s="17">
-        <f>D9-C9</f>
+        <v>18902000</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>28353000</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>-863000</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>863000</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>27490000</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>TOTALT KONSOLIDERT</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>44723691</v>
+      </c>
+      <c r="D10" s="22" t="n">
+        <v>31524851</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>47515112</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>-2791421</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <v>2791421</v>
+      </c>
+      <c r="H10" s="22" t="n">
+        <v>44723691</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>2. KONKRET TILTAKSMATRISE PER ENHET &amp; ART (SEPTEMBER - DESEMBER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Enhet</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Tiltaksbeskrivelse</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>KOSTRA-Art</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Ansvarlig Leder</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Månedlig Takt (kr)</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Total Effekt T3 (kr)</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Styringsmessig Forankring</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Slettheia</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Totalstopp for eksterne vikarbyråer (Adecco/Dedicate); overgang til intern pool</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>127040</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Enhetsleder</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Rammeavtalebehov avslått</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Slettheia</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Turnusomlegging &amp; forhåndsavtalt helgedekning, kutt i kveld/nattillegg</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>102030/31</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Avdelingsleder</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="n">
+        <v>110000</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>440000</v>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Drøftet med tillitsvalgte</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Slettheia</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Restriktiv overtidskontroll &amp; ledergodkjenning før ekstra vakter</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>104000</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Enhetsleder</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="n">
+        <v>95000</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <v>380000</v>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Digital timeregistrering</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Slettheia</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Intensivert sykefraværsoppfølging (IA) og full avstemming av NAV-sykepenger</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>102000/1690</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>HR / Enhetsleder</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Månedlig Altinn-avstemming</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Slettheia</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Toppfinansiering ressurskrevende tjenester for 2 beboere m/ 2:1-bemanning</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>170000</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Kommunalsjef</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="n">
+        <v>52105</v>
+      </c>
+      <c r="H21" s="24" t="n">
+        <v>208421</v>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Søknad Helse- og omsorgsdep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Mevold</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Stopp i eksterne lærervikarer; intern timebytte og ressursomdisponering</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>1020</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>Rektor</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Fagledermøte / leseplikt</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Mevold</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Timeplanoptimalisering: Sammenslåing av paralleller og kutt i ekstrahjelp</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>1030</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>Undervisningsinsp.</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="n">
+        <v>75000</v>
+      </c>
+      <c r="H23" s="24" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Timeplanlegger revidert</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Mevold</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Innkjøpsfrys på IKT-utstyr, nye læremidler, inventar og administrative driftsmidler</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>1110-1200</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>Rektor / Admin</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H24" s="24" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Kun akutt materiell tillates</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Mevold</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Aktiv purring og full avstemming av utestående NAV sykelønnsrefusjoner</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>1690</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Skolesekretær/HR</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="n">
+        <v>62500</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <v>250000</v>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>NAV forvaltning avstemt</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Mevold</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Samordning av spesialpedagogiske timer og assistentressurser på tvers av trinn</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>1010</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Avdelingsleder</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>41500</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <v>166000</v>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>PPT og skolehelsetjeneste</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>TOTALT</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>SAMLET REALISERT TILTAKSEFFEKT I T3</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="22">
+        <f>SUM(G17:G26)</f>
         <v/>
       </c>
-      <c r="F9" s="17" t="n">
-        <v>5896454</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>17233691</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I9" s="17">
-        <f>D9+F9+(E9*H9)</f>
+      <c r="H27" s="22">
+        <f>SUM(H17:H26)</f>
         <v/>
       </c>
-      <c r="J9" s="18">
-        <f>I9-G9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>SFO-avdelingene (Oppvekst)</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="n">
-        <v>813000</v>
-      </c>
-      <c r="D10" s="17" t="n">
-        <v>1007000</v>
-      </c>
-      <c r="E10" s="17">
-        <f>D10-C10</f>
-        <v/>
-      </c>
-      <c r="F10" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="17" t="n">
-        <v>813000</v>
-      </c>
-      <c r="H10" s="19" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I10" s="17">
-        <f>D10+F10+(E10*H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="18">
-        <f>I10-G10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Skoleskyss / Sentral stab</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="n">
-        <v>516000</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>581000</v>
-      </c>
-      <c r="E11" s="17">
-        <f>D11-C11</f>
-        <v/>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="17" t="n">
-        <v>516000</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I11" s="17">
-        <f>D11+F11+(E11*H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="18">
-        <f>I11-G11</f>
-        <v/>
+      <c r="I27" s="20" t="inlineStr">
+        <is>
+          <t>Garanterer 0 kr i avvik (Net Zero) ✓</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>